<commit_message>
Regenerate all 24 workbooks on the audit-2 fixes (incl. otc book)
Full rebuild (24/24, no failures) from the audit-2-corrected master:
- Value-Unlock family DQ-gated at the source (DDI/NNDM/PXLW/ACON no longer
  in the tab)
- _not_warrant no longer falsely demotes 4-char common stocks (Charter,
  Netgear, Comscore, Clarus, Pixelworks restored to the net-net/adjusted-P/B
  tabs where they qualify)
- Quality Net-Nets carries a $20M size floor (zombie shells gone)
- DQ EBITDA>2x-revenue leg operating-only (68 false demotions released)
- REIT add-back only where property >= 20% of assets
- otc_archetype_book rebuilt (it had been omitted from the regen and gone
  stale); the 10 generator-less legacy books are removed.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_nms_book.xlsx
+++ b/asymmetry_nms_book.xlsx
@@ -32817,12 +32817,12 @@
       </c>
       <c r="C16" s="28" t="inlineStr">
         <is>
-          <t>BANL</t>
+          <t>SCYX</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
         <is>
-          <t>Cbl International Limited</t>
+          <t>SCYNEXIS, Inc.</t>
         </is>
       </c>
       <c r="E16" s="19" t="inlineStr">
@@ -32832,12 +32832,12 @@
       </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="G16" s="20" t="inlineStr">
         <is>
-          <t>Oil, Gas &amp; Consumable Fuels</t>
+          <t>Pharmaceuticals</t>
         </is>
       </c>
       <c r="H16" s="21" t="inlineStr">
@@ -32846,7 +32846,7 @@
         </is>
       </c>
       <c r="I16" s="22" t="n">
-        <v>12457237</v>
+        <v>48653588</v>
       </c>
       <c r="J16" s="26" t="inlineStr">
         <is>
@@ -32854,23 +32854,21 @@
         </is>
       </c>
       <c r="K16" s="24" t="n">
-        <v>0.8164227183294704</v>
+        <v>0.8081594299047473</v>
       </c>
       <c r="L16" s="24" t="n">
-        <v>0.571</v>
+        <v>1</v>
       </c>
       <c r="M16" s="24" t="n">
-        <v>0.58659774</v>
+        <v>0.7269213</v>
       </c>
       <c r="N16" s="27" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="O16" s="27" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="O16" s="24" t="n">
+        <v>2.5319312</v>
       </c>
     </row>
     <row r="17" ht="17" customHeight="1">
@@ -32879,12 +32877,12 @@
       </c>
       <c r="C17" s="28" t="inlineStr">
         <is>
-          <t>SCYX</t>
+          <t>BANL</t>
         </is>
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>SCYNEXIS, Inc.</t>
+          <t>Cbl International Limited</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
@@ -32894,12 +32892,12 @@
       </c>
       <c r="F17" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="G17" s="20" t="inlineStr">
         <is>
-          <t>Pharmaceuticals</t>
+          <t>Oil, Gas &amp; Consumable Fuels</t>
         </is>
       </c>
       <c r="H17" s="21" t="inlineStr">
@@ -32908,7 +32906,7 @@
         </is>
       </c>
       <c r="I17" s="22" t="n">
-        <v>48653588</v>
+        <v>12457237</v>
       </c>
       <c r="J17" s="26" t="inlineStr">
         <is>
@@ -32916,21 +32914,23 @@
         </is>
       </c>
       <c r="K17" s="24" t="n">
-        <v>0.8081594299047473</v>
+        <v>0.8068747010339026</v>
       </c>
       <c r="L17" s="24" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="M17" s="24" t="n">
-        <v>0.7269213</v>
+        <v>0.58659774</v>
       </c>
       <c r="N17" s="27" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="O17" s="24" t="n">
-        <v>2.5319312</v>
+      <c r="O17" s="27" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
     </row>
     <row r="18" ht="17" customHeight="1">
@@ -32976,10 +32976,10 @@
         </is>
       </c>
       <c r="K18" s="24" t="n">
-        <v>0.8062111750244484</v>
+        <v>0.802895071145605</v>
       </c>
       <c r="L18" s="24" t="n">
-        <v>0.828</v>
+        <v>0.803</v>
       </c>
       <c r="M18" s="24" t="n">
         <v>0.2320380985386871</v>
@@ -51801,10 +51801,10 @@
         </is>
       </c>
       <c r="K7" s="24" t="n">
-        <v>0.7483747819327972</v>
+        <v>0.7397178222661022</v>
       </c>
       <c r="L7" s="24" t="n">
-        <v>0.667</v>
+        <v>0.6</v>
       </c>
       <c r="M7" s="27" t="inlineStr">
         <is>
@@ -65023,10 +65023,10 @@
         </is>
       </c>
       <c r="K11" s="24" t="n">
-        <v>0.6223828899889503</v>
+        <v>0.619711718787281</v>
       </c>
       <c r="L11" s="24" t="n">
-        <v>0.825</v>
+        <v>0.8</v>
       </c>
       <c r="M11" s="24" t="n">
         <v>0.9437919</v>
@@ -65259,10 +65259,10 @@
         </is>
       </c>
       <c r="K15" s="24" t="n">
-        <v>0.578025607501778</v>
+        <v>0.5742798753931376</v>
       </c>
       <c r="L15" s="24" t="n">
-        <v>0.739</v>
+        <v>0.701</v>
       </c>
       <c r="M15" s="24" t="n">
         <v>0.33102494</v>
@@ -65553,10 +65553,10 @@
         </is>
       </c>
       <c r="K20" s="24" t="n">
-        <v>0.555827069716932</v>
+        <v>0.5520472864940897</v>
       </c>
       <c r="L20" s="24" t="n">
-        <v>0.588</v>
+        <v>0.55</v>
       </c>
       <c r="M20" s="24" t="n">
         <v>0.7176173</v>

</xml_diff>

<commit_message>
Rebuild all 24 books (partial FMP segments); 13F run complete (18,515 names)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_nms_book.xlsx
+++ b/asymmetry_nms_book.xlsx
@@ -52122,36 +52122,36 @@
       </c>
       <c r="C13" s="28" t="inlineStr">
         <is>
-          <t>SKAND.OL</t>
+          <t>PRIC-B.ST</t>
         </is>
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>Skandia GreenPower AS</t>
+          <t>Pricer AB (publ)</t>
         </is>
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="F13" s="20" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="G13" s="20" t="inlineStr">
         <is>
-          <t>Independent Power and Renewable Electricity Producers</t>
+          <t>Commercial Services &amp; Supplies</t>
         </is>
       </c>
       <c r="H13" s="21" t="inlineStr">
         <is>
-          <t>Nano Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
       <c r="I13" s="22" t="n">
-        <v>19848335.28486846</v>
+        <v>68830954.20963286</v>
       </c>
       <c r="J13" s="26" t="inlineStr">
         <is>
@@ -52159,19 +52159,21 @@
         </is>
       </c>
       <c r="K13" s="24" t="n">
-        <v>0.5611153957437102</v>
+        <v>0.5636755923274757</v>
       </c>
       <c r="L13" s="24" t="n">
         <v>1</v>
       </c>
       <c r="M13" s="24" t="n">
-        <v>1.8742586</v>
-      </c>
-      <c r="N13" s="25" t="n">
-        <v>3.94</v>
+        <v>0.58504397</v>
+      </c>
+      <c r="N13" s="27" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="O13" s="24" t="n">
-        <v>0.2493113</v>
+        <v>0.30395496</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -52180,27 +52182,27 @@
       </c>
       <c r="C14" s="28" t="inlineStr">
         <is>
-          <t>CEMAT.CO</t>
+          <t>SKAND.OL</t>
         </is>
       </c>
       <c r="D14" s="18" t="inlineStr">
         <is>
-          <t>Cemat A/S</t>
+          <t>Skandia GreenPower AS</t>
         </is>
       </c>
       <c r="E14" s="19" t="inlineStr">
         <is>
-          <t>DK</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F14" s="20" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G14" s="20" t="inlineStr">
         <is>
-          <t>Real Estate Management &amp; Development</t>
+          <t>Independent Power and Renewable Electricity Producers</t>
         </is>
       </c>
       <c r="H14" s="21" t="inlineStr">
@@ -52209,29 +52211,27 @@
         </is>
       </c>
       <c r="I14" s="22" t="n">
-        <v>33402859.47088336</v>
-      </c>
-      <c r="J14" s="19" t="inlineStr">
-        <is>
-          <t>YELLOW</t>
+        <v>19848335.28486846</v>
+      </c>
+      <c r="J14" s="26" t="inlineStr">
+        <is>
+          <t>UNRESEARCHED</t>
         </is>
       </c>
       <c r="K14" s="24" t="n">
-        <v>0.5566654665206502</v>
+        <v>0.5611153957437102</v>
       </c>
       <c r="L14" s="24" t="n">
-        <v>0.989</v>
+        <v>1</v>
       </c>
       <c r="M14" s="24" t="n">
-        <v>0.9039666</v>
-      </c>
-      <c r="N14" s="27" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>1.8742586</v>
+      </c>
+      <c r="N14" s="25" t="n">
+        <v>3.94</v>
       </c>
       <c r="O14" s="24" t="n">
-        <v>1.1935964</v>
+        <v>0.2493113</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -52240,27 +52240,27 @@
       </c>
       <c r="C15" s="28" t="inlineStr">
         <is>
-          <t>GGEO.ST</t>
+          <t>CEMAT.CO</t>
         </is>
       </c>
       <c r="D15" s="18" t="inlineStr">
         <is>
-          <t>Guideline Geo AB (publ)</t>
+          <t>Cemat A/S</t>
         </is>
       </c>
       <c r="E15" s="19" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>DK</t>
         </is>
       </c>
       <c r="F15" s="20" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="G15" s="20" t="inlineStr">
         <is>
-          <t>Energy Equipment &amp; Services</t>
+          <t>Real Estate Management &amp; Development</t>
         </is>
       </c>
       <c r="H15" s="21" t="inlineStr">
@@ -52269,21 +52269,21 @@
         </is>
       </c>
       <c r="I15" s="22" t="n">
-        <v>10613705.88981759</v>
-      </c>
-      <c r="J15" s="26" t="inlineStr">
-        <is>
-          <t>UNRESEARCHED</t>
+        <v>33402859.47088336</v>
+      </c>
+      <c r="J15" s="19" t="inlineStr">
+        <is>
+          <t>YELLOW</t>
         </is>
       </c>
       <c r="K15" s="24" t="n">
-        <v>0.5558207726676844</v>
+        <v>0.5566654665206502</v>
       </c>
       <c r="L15" s="24" t="n">
-        <v>0.625</v>
+        <v>0.989</v>
       </c>
       <c r="M15" s="24" t="n">
-        <v>0.7455325</v>
+        <v>0.9039666</v>
       </c>
       <c r="N15" s="27" t="inlineStr">
         <is>
@@ -52291,7 +52291,7 @@
         </is>
       </c>
       <c r="O15" s="24" t="n">
-        <v>0.47706202</v>
+        <v>1.1935964</v>
       </c>
     </row>
     <row r="16" ht="17" customHeight="1">
@@ -52300,12 +52300,12 @@
       </c>
       <c r="C16" s="28" t="inlineStr">
         <is>
-          <t>PRIC-B.ST</t>
+          <t>GGEO.ST</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
         <is>
-          <t>Pricer AB (publ)</t>
+          <t>Guideline Geo AB (publ)</t>
         </is>
       </c>
       <c r="E16" s="19" t="inlineStr">
@@ -52315,21 +52315,21 @@
       </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="G16" s="20" t="inlineStr">
         <is>
-          <t>Commercial Services &amp; Supplies</t>
+          <t>Energy Equipment &amp; Services</t>
         </is>
       </c>
       <c r="H16" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
       <c r="I16" s="22" t="n">
-        <v>68830954.20963286</v>
+        <v>10613705.88981759</v>
       </c>
       <c r="J16" s="26" t="inlineStr">
         <is>
@@ -52337,13 +52337,13 @@
         </is>
       </c>
       <c r="K16" s="24" t="n">
-        <v>0.5544350088466974</v>
+        <v>0.5558207726676844</v>
       </c>
       <c r="L16" s="24" t="n">
-        <v>1</v>
+        <v>0.625</v>
       </c>
       <c r="M16" s="24" t="n">
-        <v>0.58504397</v>
+        <v>0.7455325</v>
       </c>
       <c r="N16" s="27" t="inlineStr">
         <is>
@@ -52351,7 +52351,7 @@
         </is>
       </c>
       <c r="O16" s="24" t="n">
-        <v>0.30395496</v>
+        <v>0.47706202</v>
       </c>
     </row>
     <row r="17" ht="17" customHeight="1">
@@ -59139,36 +59139,34 @@
       </c>
       <c r="C22" s="28" t="inlineStr">
         <is>
-          <t>GEST.MC</t>
+          <t>ELSTR.AT</t>
         </is>
       </c>
       <c r="D22" s="18" t="inlineStr">
         <is>
-          <t>Gestamp Automocion S.A.</t>
+          <t>Elastron S.A. - Steel Service Centers</t>
         </is>
       </c>
       <c r="E22" s="19" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>GR</t>
         </is>
       </c>
       <c r="F22" s="20" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="G22" s="20" t="inlineStr">
-        <is>
-          <t>Auto Components</t>
-        </is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="G22" s="20" t="n">
+        <v/>
       </c>
       <c r="H22" s="21" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
       <c r="I22" s="22" t="n">
-        <v>1939274358.011536</v>
+        <v>54860998.78386497</v>
       </c>
       <c r="J22" s="26" t="inlineStr">
         <is>
@@ -59176,19 +59174,19 @@
         </is>
       </c>
       <c r="K22" s="24" t="n">
-        <v>0.4601482867945089</v>
+        <v>0.4659925273728007</v>
       </c>
       <c r="L22" s="24" t="n">
-        <v>0.989</v>
+        <v>0.778</v>
       </c>
       <c r="M22" s="24" t="n">
-        <v>0.7032365</v>
+        <v>0.5548496000000001</v>
       </c>
       <c r="N22" s="25" t="n">
-        <v>2.8499998</v>
+        <v>3.95</v>
       </c>
       <c r="O22" s="24" t="n">
-        <v>0.1474581</v>
+        <v>0.28365088</v>
       </c>
     </row>
     <row r="23" ht="17" customHeight="1">
@@ -59197,34 +59195,36 @@
       </c>
       <c r="C23" s="28" t="inlineStr">
         <is>
-          <t>ELSTR.AT</t>
+          <t>GEST.MC</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
         <is>
-          <t>Elastron S.A. - Steel Service Centers</t>
+          <t>Gestamp Automocion S.A.</t>
         </is>
       </c>
       <c r="E23" s="19" t="inlineStr">
         <is>
-          <t>GR</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="F23" s="20" t="inlineStr">
         <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="G23" s="20" t="n">
-        <v/>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="G23" s="20" t="inlineStr">
+        <is>
+          <t>Auto Components</t>
+        </is>
       </c>
       <c r="H23" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Small Cap</t>
         </is>
       </c>
       <c r="I23" s="22" t="n">
-        <v>54860998.78386497</v>
+        <v>1939274358.011536</v>
       </c>
       <c r="J23" s="26" t="inlineStr">
         <is>
@@ -59232,19 +59232,19 @@
         </is>
       </c>
       <c r="K23" s="24" t="n">
-        <v>0.4595375877517608</v>
+        <v>0.4601482867945089</v>
       </c>
       <c r="L23" s="24" t="n">
-        <v>0.778</v>
+        <v>0.989</v>
       </c>
       <c r="M23" s="24" t="n">
-        <v>0.5548496000000001</v>
+        <v>0.7032365</v>
       </c>
       <c r="N23" s="25" t="n">
-        <v>3.95</v>
+        <v>2.8499998</v>
       </c>
       <c r="O23" s="24" t="n">
-        <v>0.28365088</v>
+        <v>0.1474581</v>
       </c>
     </row>
     <row r="24" ht="17" customHeight="1">

</xml_diff>